<commit_message>
Update Valkyrie V2 HT100 Build Guide Beta.xlsx
</commit_message>
<xml_diff>
--- a/V2 BETA/BOM/Valkyrie V2 HT100 Build Guide Beta.xlsx
+++ b/V2 BETA/BOM/Valkyrie V2 HT100 Build Guide Beta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3837cd5b4a1a02ac/Document Library/GitHub/Project-Valkyrie/V2 BETA/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4170" documentId="8_{5107759B-8870-48A8-933E-C4A7F6F41B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C67DEFA-BB35-4EB6-B932-3884EAFA3343}"/>
+  <xr:revisionPtr revIDLastSave="4175" documentId="8_{5107759B-8870-48A8-933E-C4A7F6F41B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC4C0134-8ED1-434E-A067-5F4EFABFA36A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2093" uniqueCount="1198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2090" uniqueCount="1195">
   <si>
     <t>Type</t>
   </si>
@@ -2222,15 +2222,6 @@
     <t>Drop off the flint zone probe</t>
   </si>
   <si>
-    <t>tool_Hd_xxxxx</t>
-  </si>
-  <si>
-    <t>tool change file</t>
-  </si>
-  <si>
-    <t>Optional - Settings required for each tool</t>
-  </si>
-  <si>
     <t>z_offset</t>
   </si>
   <si>
@@ -2346,12 +2337,6 @@
   </si>
   <si>
     <t>This macro is run when a print has "100%"  completed</t>
-  </si>
-  <si>
-    <t>tool.g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional- Define tool perameters set by the tool_hd_x .g  file </t>
   </si>
   <si>
     <t>Machine Gcode</t>
@@ -3712,6 +3697,12 @@
   </si>
   <si>
     <t>chamber_ramp</t>
+  </si>
+  <si>
+    <t>Ramp up chamber temp</t>
+  </si>
+  <si>
+    <t>To avoid heater faults</t>
   </si>
 </sst>
 </file>
@@ -7799,10 +7790,10 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{08A74962-DE02-40B7-84D1-EBA03C7907E7}" name="Table3" displayName="Table3" ref="A1:C13" totalsRowShown="0">
-  <autoFilter ref="A1:C13" xr:uid="{08A74962-DE02-40B7-84D1-EBA03C7907E7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C13">
-    <sortCondition ref="A1:A13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{08A74962-DE02-40B7-84D1-EBA03C7907E7}" name="Table3" displayName="Table3" ref="A1:C12" totalsRowShown="0">
+  <autoFilter ref="A1:C12" xr:uid="{08A74962-DE02-40B7-84D1-EBA03C7907E7}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C12">
+    <sortCondition ref="A1:A12"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="5" xr3:uid="{8D8B2F09-EE52-45AA-BAA6-D22E0DE184E9}" name="Macro" dataDxfId="18"/>
@@ -7814,10 +7805,10 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{22CC0901-A1E8-42BF-83D2-CD8909D9E84D}" name="Table4" displayName="Table4" ref="A16:C33" totalsRowShown="0">
-  <autoFilter ref="A16:C33" xr:uid="{22CC0901-A1E8-42BF-83D2-CD8909D9E84D}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A17:C33">
-    <sortCondition ref="A16:A33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{22CC0901-A1E8-42BF-83D2-CD8909D9E84D}" name="Table4" displayName="Table4" ref="A15:C31" totalsRowShown="0">
+  <autoFilter ref="A15:C31" xr:uid="{22CC0901-A1E8-42BF-83D2-CD8909D9E84D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A16:C31">
+    <sortCondition ref="A15:A31"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="2" xr3:uid="{72E39D2F-151A-44B2-BA84-B7F34C14C282}" name="System" dataDxfId="17"/>
@@ -7829,8 +7820,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{65AAB1FE-3FF5-4932-83DF-59F4C29F97F6}" name="Table5" displayName="Table5" ref="A35:B39" totalsRowShown="0">
-  <autoFilter ref="A35:B39" xr:uid="{65AAB1FE-3FF5-4932-83DF-59F4C29F97F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{65AAB1FE-3FF5-4932-83DF-59F4C29F97F6}" name="Table5" displayName="Table5" ref="A33:B37" totalsRowShown="0">
+  <autoFilter ref="A33:B37" xr:uid="{65AAB1FE-3FF5-4932-83DF-59F4C29F97F6}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{9B5CA5FD-9D48-460B-8000-5A3DECA0A58C}" name="Machine Gcode"/>
     <tableColumn id="3" xr3:uid="{122CB247-7719-4458-B0BE-E37243F62675}" name="Description"/>
@@ -7840,10 +7831,10 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{255B9BA2-9874-4909-AB93-96FB850EFBDB}" name="Table58" displayName="Table58" ref="A44:B54" totalsRowShown="0">
-  <autoFilter ref="A44:B54" xr:uid="{255B9BA2-9874-4909-AB93-96FB850EFBDB}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A45:B54">
-    <sortCondition ref="A44:A54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{255B9BA2-9874-4909-AB93-96FB850EFBDB}" name="Table58" displayName="Table58" ref="A42:B52" totalsRowShown="0">
+  <autoFilter ref="A42:B52" xr:uid="{255B9BA2-9874-4909-AB93-96FB850EFBDB}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A43:B52">
+    <sortCondition ref="A42:A52"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{646EABC4-F408-4AD0-8ED9-44B19D7B9F30}" name="Filaments"/>
@@ -15235,7 +15226,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -15260,7 +15251,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>1197</v>
+        <v>1192</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1194</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -15366,94 +15363,94 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="147" t="s">
+      <c r="A12" s="25" t="s">
         <v>720</v>
       </c>
-      <c r="B12" s="146" t="s">
+      <c r="B12" t="s">
         <v>721</v>
       </c>
-      <c r="C12" s="148" t="s">
+      <c r="C12" t="s">
         <v>722</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="25" t="s">
-        <v>723</v>
-      </c>
-      <c r="B13" t="s">
-        <v>724</v>
-      </c>
-      <c r="C13" t="s">
-        <v>725</v>
-      </c>
+      <c r="A13" s="25"/>
+      <c r="B13" s="25"/>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="25"/>
       <c r="B14" s="25"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
+      <c r="A15" s="65" t="s">
+        <v>649</v>
+      </c>
+      <c r="B15" t="s">
+        <v>723</v>
+      </c>
+      <c r="C15" t="s">
+        <v>361</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="65" t="s">
-        <v>649</v>
+      <c r="A16" s="25" t="s">
+        <v>724</v>
       </c>
       <c r="B16" t="s">
+        <v>725</v>
+      </c>
+      <c r="C16" t="s">
         <v>726</v>
-      </c>
-      <c r="C16" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="25" t="s">
         <v>727</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" s="4" t="s">
         <v>728</v>
-      </c>
-      <c r="C17" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="25" t="s">
+        <v>729</v>
+      </c>
+      <c r="C18" t="s">
         <v>730</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>731</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="25" t="s">
+        <v>731</v>
+      </c>
+      <c r="C19" t="s">
         <v>732</v>
-      </c>
-      <c r="C19" t="s">
-        <v>733</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="25" t="s">
+        <v>733</v>
+      </c>
+      <c r="C20" t="s">
         <v>734</v>
-      </c>
-      <c r="C20" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="25" t="s">
+        <v>735</v>
+      </c>
+      <c r="C21" t="s">
         <v>736</v>
-      </c>
-      <c r="C21" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="C22" t="s">
         <v>738</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" s="134" t="s">
         <v>739</v>
       </c>
     </row>
@@ -15461,10 +15458,10 @@
       <c r="A23" s="25" t="s">
         <v>740</v>
       </c>
+      <c r="B23" t="s">
+        <v>741</v>
+      </c>
       <c r="C23" t="s">
-        <v>741</v>
-      </c>
-      <c r="E23" s="134" t="s">
         <v>742</v>
       </c>
     </row>
@@ -15472,31 +15469,31 @@
       <c r="A24" s="25" t="s">
         <v>743</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>744</v>
-      </c>
-      <c r="C24" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="25" t="s">
+        <v>745</v>
+      </c>
+      <c r="C25" t="s">
         <v>746</v>
-      </c>
-      <c r="C25" t="s">
-        <v>747</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="25" t="s">
+        <v>747</v>
+      </c>
+      <c r="C26" t="s">
         <v>748</v>
-      </c>
-      <c r="C26" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="25" t="s">
+        <v>749</v>
+      </c>
+      <c r="B27" t="s">
         <v>750</v>
       </c>
       <c r="C27" t="s">
@@ -15518,185 +15515,166 @@
       <c r="A29" s="25" t="s">
         <v>755</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>756</v>
-      </c>
-      <c r="C29" t="s">
-        <v>757</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="25" t="s">
+        <v>757</v>
+      </c>
+      <c r="C30" t="s">
         <v>758</v>
       </c>
-      <c r="C30" t="s">
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="25"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="B32" s="25"/>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="47" t="s">
         <v>759</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="25" t="s">
+      <c r="B33" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
         <v>760</v>
       </c>
-      <c r="C31" t="s">
+      <c r="B34" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="147" t="s">
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
         <v>762</v>
       </c>
-      <c r="C32" s="148" t="s">
-        <v>763</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="25"/>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="B34" s="25"/>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="47" t="s">
-        <v>764</v>
-      </c>
       <c r="B35" t="s">
-        <v>361</v>
+        <v>761</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B36" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
+        <v>764</v>
+      </c>
+      <c r="B37" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="B39" t="s">
+        <v>765</v>
+      </c>
+      <c r="D39" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="B40" t="s">
         <v>767</v>
       </c>
-      <c r="B37" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
+      <c r="D40" t="s">
         <v>768</v>
       </c>
-      <c r="B38" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="47" t="s">
         <v>769</v>
       </c>
-      <c r="B39" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="B41" t="s">
+      <c r="B42" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
         <v>770</v>
       </c>
-      <c r="D41" t="s">
+      <c r="B43" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="B42" t="s">
-        <v>772</v>
-      </c>
-      <c r="D42" t="s">
-        <v>773</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="47" t="s">
-        <v>774</v>
-      </c>
       <c r="B44" t="s">
-        <v>361</v>
+        <v>761</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="B45" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B46" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B47" t="s">
-        <v>778</v>
+        <v>761</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="B48" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="B49" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B50" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="B51" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="B52" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
-        <v>784</v>
-      </c>
-      <c r="B53" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
-        <v>785</v>
-      </c>
-      <c r="B54" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
   </sheetData>
@@ -15737,14 +15715,14 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1">
       <c r="A1" s="107" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="B1" s="105"/>
       <c r="C1" s="105"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1">
       <c r="A2" s="108" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="B2" s="105"/>
       <c r="C2" s="105"/>
@@ -15754,80 +15732,80 @@
       <c r="B3" s="128"/>
       <c r="C3" s="128"/>
       <c r="D3" s="110" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="E3" s="110" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="F3" s="110" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="G3" s="110" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="H3" s="110" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="I3" s="110" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="J3" s="133" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="K3" s="110" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="L3" s="112" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
     </row>
     <row r="4" spans="1:12" s="106" customFormat="1" ht="46.5" customHeight="1" thickBot="1">
       <c r="A4" s="126" t="s">
+        <v>788</v>
+      </c>
+      <c r="B4" s="126" t="s">
+        <v>789</v>
+      </c>
+      <c r="C4" s="126" t="s">
+        <v>790</v>
+      </c>
+      <c r="D4" s="126" t="s">
+        <v>791</v>
+      </c>
+      <c r="E4" s="126" t="s">
+        <v>792</v>
+      </c>
+      <c r="F4" s="126" t="s">
         <v>793</v>
       </c>
-      <c r="B4" s="126" t="s">
+      <c r="G4" s="126" t="s">
         <v>794</v>
       </c>
-      <c r="C4" s="126" t="s">
+      <c r="H4" s="126" t="s">
         <v>795</v>
       </c>
-      <c r="D4" s="126" t="s">
+      <c r="I4" s="126" t="s">
         <v>796</v>
       </c>
-      <c r="E4" s="126" t="s">
+      <c r="J4" s="126" t="s">
         <v>797</v>
       </c>
-      <c r="F4" s="126" t="s">
+      <c r="K4" s="126" t="s">
         <v>798</v>
       </c>
-      <c r="G4" s="126" t="s">
+      <c r="L4" s="126" t="s">
         <v>799</v>
-      </c>
-      <c r="H4" s="126" t="s">
-        <v>800</v>
-      </c>
-      <c r="I4" s="126" t="s">
-        <v>801</v>
-      </c>
-      <c r="J4" s="126" t="s">
-        <v>802</v>
-      </c>
-      <c r="K4" s="126" t="s">
-        <v>803</v>
-      </c>
-      <c r="L4" s="126" t="s">
-        <v>804</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A5" s="129" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="B5" s="122" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C5" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D5" s="123">
         <v>105</v>
@@ -15859,13 +15837,13 @@
     </row>
     <row r="6" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A6" s="129" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="B6" s="122" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C6" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D6" s="123">
         <v>105</v>
@@ -15897,13 +15875,13 @@
     </row>
     <row r="7" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A7" s="129" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="B7" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C7" s="123" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="D7" s="123">
         <v>90</v>
@@ -15935,10 +15913,10 @@
     </row>
     <row r="8" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A8" s="129" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="B8" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C8" s="123">
         <v>0</v>
@@ -15956,10 +15934,10 @@
         <v>50</v>
       </c>
       <c r="H8" s="123" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="I8" s="124" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="J8" s="123">
         <v>80</v>
@@ -15973,13 +15951,13 @@
     </row>
     <row r="9" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A9" s="121" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="B9" s="122" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="C9" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D9" s="123">
         <v>105</v>
@@ -16011,13 +15989,13 @@
     </row>
     <row r="10" spans="1:12" s="106" customFormat="1" ht="17.25" customHeight="1">
       <c r="A10" s="121" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="B10" s="122" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="C10" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D10" s="123">
         <v>60</v>
@@ -16049,13 +16027,13 @@
     </row>
     <row r="11" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A11" s="121" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="B11" s="122" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="C11" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D11" s="123">
         <v>60</v>
@@ -16087,13 +16065,13 @@
     </row>
     <row r="12" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="121" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="B12" s="122" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="C12" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D12" s="123">
         <v>60</v>
@@ -16125,13 +16103,13 @@
     </row>
     <row r="13" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A13" s="121" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="B13" s="122" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="C13" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D13" s="123">
         <v>70</v>
@@ -16163,10 +16141,10 @@
     </row>
     <row r="14" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A14" s="121" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="B14" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C14" s="123">
         <v>0</v>
@@ -16201,11 +16179,11 @@
     </row>
     <row r="15" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A15" s="129" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="B15" s="122"/>
       <c r="C15" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D15" s="123">
         <v>137</v>
@@ -16237,11 +16215,11 @@
     </row>
     <row r="16" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A16" s="129" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="B16" s="122"/>
       <c r="C16" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D16" s="123">
         <v>126</v>
@@ -16273,13 +16251,13 @@
     </row>
     <row r="17" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A17" s="121" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="B17" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C17" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D17" s="123">
         <v>145</v>
@@ -16311,13 +16289,13 @@
     </row>
     <row r="18" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A18" s="121" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
       <c r="B18" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C18" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D18" s="123">
         <v>113</v>
@@ -16349,11 +16327,11 @@
     </row>
     <row r="19" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A19" s="121" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="B19" s="122"/>
       <c r="C19" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D19" s="123">
         <v>158</v>
@@ -16385,11 +16363,11 @@
     </row>
     <row r="20" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A20" s="121" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="B20" s="122"/>
       <c r="C20" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D20" s="123">
         <v>143</v>
@@ -16425,7 +16403,7 @@
       </c>
       <c r="B21" s="122"/>
       <c r="C21" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D21" s="123">
         <v>140</v>
@@ -16457,13 +16435,13 @@
     </row>
     <row r="22" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A22" s="121" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="B22" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C22" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D22" s="123">
         <v>113</v>
@@ -16495,13 +16473,13 @@
     </row>
     <row r="23" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A23" s="129" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="B23" s="122" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="C23" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D23" s="123">
         <v>143</v>
@@ -16533,13 +16511,13 @@
     </row>
     <row r="24" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A24" s="129" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="B24" s="122" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="C24" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D24" s="123">
         <v>165</v>
@@ -16571,13 +16549,13 @@
     </row>
     <row r="25" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A25" s="121" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="B25" s="122" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="C25" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D25" s="123">
         <v>165</v>
@@ -16609,13 +16587,13 @@
     </row>
     <row r="26" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A26" s="130" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="B26" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C26" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D26" s="123">
         <v>70</v>
@@ -16647,13 +16625,13 @@
     </row>
     <row r="27" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A27" s="129" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="B27" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C27" s="123" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="D27" s="123">
         <v>80</v>
@@ -16685,13 +16663,13 @@
     </row>
     <row r="28" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A28" s="129" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
       <c r="B28" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C28" s="123" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="D28" s="123">
         <v>85</v>
@@ -16726,10 +16704,10 @@
         <v>664</v>
       </c>
       <c r="B29" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C29" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D29" s="123">
         <v>90</v>
@@ -16761,10 +16739,10 @@
     </row>
     <row r="30" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A30" s="129" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="B30" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C30" s="123">
         <v>0</v>
@@ -16802,7 +16780,7 @@
         <v>663</v>
       </c>
       <c r="B31" s="122" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C31" s="123">
         <v>0</v>
@@ -16837,10 +16815,10 @@
     </row>
     <row r="32" spans="1:12" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A32" s="129" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="B32" s="122" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="C32" s="123">
         <v>0</v>
@@ -16875,10 +16853,10 @@
     </row>
     <row r="33" spans="1:13" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A33" s="129" t="s">
-        <v>836</v>
+        <v>831</v>
       </c>
       <c r="B33" s="122" t="s">
-        <v>837</v>
+        <v>832</v>
       </c>
       <c r="C33" s="123">
         <v>0</v>
@@ -16913,11 +16891,11 @@
     </row>
     <row r="34" spans="1:13" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A34" s="129" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="B34" s="122"/>
       <c r="C34" s="123" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D34" s="123">
         <v>170</v>
@@ -16932,10 +16910,10 @@
         <v>100</v>
       </c>
       <c r="H34" s="123" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="I34" s="124" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="J34" s="123">
         <v>158</v>
@@ -16949,11 +16927,11 @@
     </row>
     <row r="35" spans="1:13" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A35" s="129" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="B35" s="122"/>
       <c r="C35" s="123" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="D35" s="123">
         <v>80</v>
@@ -16985,10 +16963,10 @@
     </row>
     <row r="36" spans="1:13" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A36" s="121" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="B36" s="122" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="C36" s="123">
         <v>0</v>
@@ -17023,7 +17001,7 @@
     </row>
     <row r="37" spans="1:13" s="106" customFormat="1" ht="15.75" customHeight="1">
       <c r="A37" s="121" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="B37" s="122"/>
       <c r="C37" s="123">
@@ -17074,7 +17052,7 @@
     </row>
     <row r="39" spans="1:13" ht="15.75" customHeight="1">
       <c r="A39" s="109" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="B39" s="229"/>
       <c r="C39" s="229"/>
@@ -17091,7 +17069,7 @@
     </row>
     <row r="41" spans="1:13" ht="15.75" customHeight="1">
       <c r="A41" s="109" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="B41" s="270"/>
       <c r="C41" s="270"/>
@@ -17107,7 +17085,7 @@
     </row>
     <row r="42" spans="1:13" ht="15.75" customHeight="1">
       <c r="A42" s="229" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="B42" s="105"/>
       <c r="C42" s="105"/>
@@ -17116,7 +17094,7 @@
     </row>
     <row r="43" spans="1:13" ht="15.75" customHeight="1">
       <c r="A43" s="229" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="B43" s="105"/>
       <c r="C43" s="105"/>
@@ -17125,7 +17103,7 @@
     </row>
     <row r="44" spans="1:13" ht="15.75" customHeight="1">
       <c r="A44" s="229" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="B44" s="105"/>
       <c r="C44" s="105"/>
@@ -17133,7 +17111,7 @@
     </row>
     <row r="45" spans="1:13" ht="15.75" customHeight="1">
       <c r="A45" s="229" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="B45" s="105"/>
       <c r="C45" s="105"/>
@@ -17141,7 +17119,7 @@
     </row>
     <row r="46" spans="1:13" ht="15.75" customHeight="1">
       <c r="A46" s="229" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="B46" s="105"/>
       <c r="C46" s="105"/>
@@ -17151,7 +17129,7 @@
     </row>
     <row r="47" spans="1:13" ht="15.75" customHeight="1">
       <c r="A47" s="117" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="B47" s="117"/>
       <c r="C47" s="117"/>
@@ -17177,7 +17155,7 @@
     </row>
     <row r="49" spans="1:13" ht="15.75" customHeight="1">
       <c r="A49" s="131" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="E49" s="120"/>
       <c r="F49" s="120"/>
@@ -17191,7 +17169,7 @@
     </row>
     <row r="50" spans="1:13" ht="15.75" customHeight="1">
       <c r="A50" s="131" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="E50" s="120"/>
       <c r="F50" s="120"/>
@@ -24428,7 +24406,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="102" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -24436,32 +24414,32 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="103" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="104" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="102" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="102" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="102" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="102" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -24469,17 +24447,17 @@
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="103" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="104" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="102" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -24487,37 +24465,37 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="103" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="102" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="102" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="102" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="102" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="102" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="102" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -24525,22 +24503,22 @@
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="103" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="102" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" s="102" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="102" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
     </row>
   </sheetData>
@@ -24569,39 +24547,39 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="277" t="s">
+        <v>868</v>
+      </c>
+      <c r="B1" s="278" t="s">
+        <v>869</v>
+      </c>
+      <c r="C1" s="278" t="s">
+        <v>870</v>
+      </c>
+      <c r="D1" s="278" t="s">
+        <v>871</v>
+      </c>
+      <c r="E1" s="278" t="s">
+        <v>872</v>
+      </c>
+      <c r="F1" s="278" t="s">
         <v>873</v>
       </c>
-      <c r="B1" s="278" t="s">
+      <c r="G1" s="279" t="s">
         <v>874</v>
       </c>
-      <c r="C1" s="278" t="s">
+      <c r="H1" s="274" t="s">
         <v>875</v>
       </c>
-      <c r="D1" s="278" t="s">
-        <v>876</v>
-      </c>
-      <c r="E1" s="278" t="s">
-        <v>877</v>
-      </c>
-      <c r="F1" s="278" t="s">
-        <v>878</v>
-      </c>
-      <c r="G1" s="279" t="s">
-        <v>879</v>
-      </c>
-      <c r="H1" s="274" t="s">
-        <v>880</v>
-      </c>
       <c r="J1" s="272" t="s">
-        <v>1078</v>
+        <v>1073</v>
       </c>
       <c r="K1" s="272" t="s">
-        <v>1196</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="277" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="B2" s="278">
         <v>1</v>
@@ -24619,56 +24597,56 @@
         <v>1</v>
       </c>
       <c r="G2" s="279" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="H2" s="274">
         <v>2</v>
       </c>
       <c r="J2" s="280" t="s">
-        <v>1079</v>
+        <v>1074</v>
       </c>
       <c r="K2" s="272" t="s">
-        <v>1112</v>
+        <v>1107</v>
       </c>
       <c r="L2" s="272" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="277" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="B3" s="278" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="C3" s="278" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="D3" s="281" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="E3" s="281" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="F3" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="H3" s="274" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="J3" s="280" t="s">
-        <v>1080</v>
+        <v>1075</v>
       </c>
       <c r="K3" s="272" t="s">
-        <v>1114</v>
+        <v>1109</v>
       </c>
       <c r="L3" s="272" t="s">
-        <v>1115</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="277" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="B4" s="278">
         <v>450</v>
@@ -24677,7 +24655,7 @@
         <v>450</v>
       </c>
       <c r="D4" s="278" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="E4" s="278">
         <v>285</v>
@@ -24689,33 +24667,33 @@
         <v>300</v>
       </c>
       <c r="H4" s="274" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="J4" s="280" t="s">
-        <v>1081</v>
+        <v>1076</v>
       </c>
       <c r="K4" s="272" t="s">
         <v>667</v>
       </c>
       <c r="L4" s="272" t="s">
-        <v>1116</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="277" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="B5" s="278" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="C5" s="278" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="D5" s="278">
         <v>150</v>
       </c>
       <c r="E5" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="F5" s="278">
         <v>157</v>
@@ -24724,21 +24702,21 @@
         <v>120</v>
       </c>
       <c r="H5" s="274" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="J5" s="280" t="s">
-        <v>1082</v>
+        <v>1077</v>
       </c>
       <c r="K5" s="272" t="s">
-        <v>1117</v>
+        <v>1112</v>
       </c>
       <c r="L5" s="272" t="s">
-        <v>1118</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1">
       <c r="A6" s="277" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="B6" s="278">
         <v>80</v>
@@ -24747,22 +24725,22 @@
         <v>100</v>
       </c>
       <c r="D6" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E6" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="F6" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G6" s="279">
         <v>60</v>
       </c>
       <c r="H6" s="274" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="J6" s="280" t="s">
-        <v>1083</v>
+        <v>1078</v>
       </c>
       <c r="K6" s="272" t="s">
         <v>561</v>
@@ -24770,583 +24748,583 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="277" t="s">
+        <v>891</v>
+      </c>
+      <c r="B7" s="278" t="s">
+        <v>892</v>
+      </c>
+      <c r="C7" s="278" t="s">
+        <v>893</v>
+      </c>
+      <c r="D7" s="278" t="s">
+        <v>894</v>
+      </c>
+      <c r="E7" s="278" t="s">
+        <v>895</v>
+      </c>
+      <c r="F7" s="278" t="s">
         <v>896</v>
       </c>
-      <c r="B7" s="278" t="s">
+      <c r="G7" s="279" t="s">
         <v>897</v>
       </c>
-      <c r="C7" s="278" t="s">
+      <c r="H7" s="274" t="s">
         <v>898</v>
       </c>
-      <c r="D7" s="278" t="s">
-        <v>899</v>
-      </c>
-      <c r="E7" s="278" t="s">
-        <v>900</v>
-      </c>
-      <c r="F7" s="278" t="s">
-        <v>901</v>
-      </c>
-      <c r="G7" s="279" t="s">
-        <v>902</v>
-      </c>
-      <c r="H7" s="274" t="s">
-        <v>903</v>
-      </c>
       <c r="J7" s="280" t="s">
-        <v>1084</v>
+        <v>1079</v>
       </c>
       <c r="K7" s="272" t="s">
-        <v>1119</v>
+        <v>1114</v>
       </c>
       <c r="L7" s="272" t="s">
-        <v>1120</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="277" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="B8" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="C8" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="D8" s="278" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="E8" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="F8" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="G8" s="279" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="H8" s="274" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="J8" s="280" t="s">
-        <v>1085</v>
+        <v>1080</v>
       </c>
       <c r="K8" s="272" t="s">
-        <v>1121</v>
+        <v>1116</v>
       </c>
       <c r="L8" s="272" t="s">
-        <v>1122</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="277" t="s">
+        <v>903</v>
+      </c>
+      <c r="B9" s="278" t="s">
+        <v>904</v>
+      </c>
+      <c r="C9" s="278" t="s">
+        <v>904</v>
+      </c>
+      <c r="D9" s="278" t="s">
+        <v>905</v>
+      </c>
+      <c r="E9" s="278" t="s">
+        <v>906</v>
+      </c>
+      <c r="F9" s="278" t="s">
+        <v>907</v>
+      </c>
+      <c r="H9" s="274" t="s">
         <v>908</v>
       </c>
-      <c r="B9" s="278" t="s">
-        <v>909</v>
-      </c>
-      <c r="C9" s="278" t="s">
-        <v>909</v>
-      </c>
-      <c r="D9" s="278" t="s">
-        <v>910</v>
-      </c>
-      <c r="E9" s="278" t="s">
-        <v>911</v>
-      </c>
-      <c r="F9" s="278" t="s">
-        <v>912</v>
-      </c>
-      <c r="H9" s="274" t="s">
-        <v>913</v>
-      </c>
       <c r="J9" s="280" t="s">
-        <v>1086</v>
+        <v>1081</v>
       </c>
       <c r="K9" s="272" t="s">
-        <v>1123</v>
+        <v>1118</v>
       </c>
       <c r="L9" s="272" t="s">
-        <v>1124</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1">
       <c r="A10" s="277" t="s">
+        <v>909</v>
+      </c>
+      <c r="B10" s="282" t="s">
+        <v>910</v>
+      </c>
+      <c r="C10" s="282" t="s">
+        <v>911</v>
+      </c>
+      <c r="D10" s="282" t="s">
+        <v>912</v>
+      </c>
+      <c r="E10" s="282" t="s">
+        <v>913</v>
+      </c>
+      <c r="F10" s="278" t="s">
         <v>914</v>
       </c>
-      <c r="B10" s="282" t="s">
+      <c r="G10" s="275" t="s">
         <v>915</v>
       </c>
-      <c r="C10" s="282" t="s">
+      <c r="H10" s="274" t="s">
         <v>916</v>
       </c>
-      <c r="D10" s="282" t="s">
-        <v>917</v>
-      </c>
-      <c r="E10" s="282" t="s">
-        <v>918</v>
-      </c>
-      <c r="F10" s="278" t="s">
-        <v>919</v>
-      </c>
-      <c r="G10" s="275" t="s">
-        <v>920</v>
-      </c>
-      <c r="H10" s="274" t="s">
-        <v>921</v>
-      </c>
       <c r="J10" s="280" t="s">
-        <v>1087</v>
+        <v>1082</v>
       </c>
       <c r="K10" s="272" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="277" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="B11" s="278" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="C11" s="278" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="D11" s="278" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="E11" s="278" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="F11" s="278" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="G11" s="279" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="H11" s="274" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="J11" s="280" t="s">
-        <v>1088</v>
+        <v>1083</v>
       </c>
       <c r="K11" s="272" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="L11" s="272" t="s">
-        <v>1125</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="283" t="s">
+        <v>922</v>
+      </c>
+      <c r="B12" s="282" t="s">
+        <v>923</v>
+      </c>
+      <c r="C12" s="282" t="s">
+        <v>924</v>
+      </c>
+      <c r="D12" s="284" t="s">
+        <v>925</v>
+      </c>
+      <c r="E12" s="282" t="s">
+        <v>926</v>
+      </c>
+      <c r="F12" s="284" t="s">
         <v>927</v>
       </c>
-      <c r="B12" s="282" t="s">
+      <c r="H12" s="274" t="s">
         <v>928</v>
       </c>
-      <c r="C12" s="282" t="s">
-        <v>929</v>
-      </c>
-      <c r="D12" s="284" t="s">
-        <v>930</v>
-      </c>
-      <c r="E12" s="282" t="s">
-        <v>931</v>
-      </c>
-      <c r="F12" s="284" t="s">
-        <v>932</v>
-      </c>
-      <c r="H12" s="274" t="s">
-        <v>933</v>
-      </c>
       <c r="J12" s="280" t="s">
-        <v>1089</v>
+        <v>1084</v>
       </c>
       <c r="K12" s="272" t="s">
-        <v>1126</v>
+        <v>1121</v>
       </c>
       <c r="L12" s="272" t="s">
-        <v>1127</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="277" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
       <c r="B13" s="278" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="C13" s="278" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="D13" s="278">
         <v>120</v>
       </c>
       <c r="E13" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="F13" s="278" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="G13" s="279" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="H13" s="274" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="J13" s="280" t="s">
-        <v>1090</v>
+        <v>1085</v>
       </c>
       <c r="K13" s="272" t="s">
-        <v>1128</v>
+        <v>1123</v>
       </c>
       <c r="L13" s="272" t="s">
-        <v>1129</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="277" t="s">
+        <v>933</v>
+      </c>
+      <c r="B14" s="278" t="s">
+        <v>934</v>
+      </c>
+      <c r="C14" s="278" t="s">
+        <v>934</v>
+      </c>
+      <c r="D14" s="278" t="s">
+        <v>935</v>
+      </c>
+      <c r="E14" s="278" t="s">
+        <v>936</v>
+      </c>
+      <c r="F14" s="278" t="s">
+        <v>937</v>
+      </c>
+      <c r="G14" s="279" t="s">
         <v>938</v>
       </c>
-      <c r="B14" s="278" t="s">
+      <c r="H14" s="274" t="s">
         <v>939</v>
       </c>
-      <c r="C14" s="278" t="s">
-        <v>939</v>
-      </c>
-      <c r="D14" s="278" t="s">
-        <v>940</v>
-      </c>
-      <c r="E14" s="278" t="s">
-        <v>941</v>
-      </c>
-      <c r="F14" s="278" t="s">
-        <v>942</v>
-      </c>
-      <c r="G14" s="279" t="s">
-        <v>943</v>
-      </c>
-      <c r="H14" s="274" t="s">
-        <v>944</v>
-      </c>
       <c r="J14" s="280" t="s">
-        <v>1091</v>
+        <v>1086</v>
       </c>
       <c r="K14" s="272" t="s">
-        <v>1130</v>
+        <v>1125</v>
       </c>
       <c r="L14" s="272" t="s">
-        <v>1131</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="273" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="B15" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="C15" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="H15" s="274" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="J15" s="280" t="s">
-        <v>1092</v>
+        <v>1087</v>
       </c>
       <c r="K15" s="272" t="s">
-        <v>1132</v>
+        <v>1127</v>
       </c>
       <c r="L15" s="272" t="s">
-        <v>1133</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="277" t="s">
+        <v>941</v>
+      </c>
+      <c r="B16" s="278" t="s">
+        <v>942</v>
+      </c>
+      <c r="C16" s="278" t="s">
+        <v>943</v>
+      </c>
+      <c r="D16" s="278" t="s">
+        <v>944</v>
+      </c>
+      <c r="E16" s="278" t="s">
+        <v>945</v>
+      </c>
+      <c r="F16" s="278" t="s">
+        <v>945</v>
+      </c>
+      <c r="H16" s="274" t="s">
         <v>946</v>
       </c>
-      <c r="B16" s="278" t="s">
-        <v>947</v>
-      </c>
-      <c r="C16" s="278" t="s">
-        <v>948</v>
-      </c>
-      <c r="D16" s="278" t="s">
-        <v>949</v>
-      </c>
-      <c r="E16" s="278" t="s">
-        <v>950</v>
-      </c>
-      <c r="F16" s="278" t="s">
-        <v>950</v>
-      </c>
-      <c r="H16" s="274" t="s">
-        <v>951</v>
-      </c>
       <c r="J16" s="280" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="K16" s="272" t="s">
-        <v>1134</v>
+        <v>1129</v>
       </c>
       <c r="L16" s="272" t="s">
-        <v>1135</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15" customHeight="1">
       <c r="A17" s="277" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="B17" s="278" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="C17" s="278" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="D17" s="278" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="E17" s="278" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="F17" s="278" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="H17" s="274" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="J17" s="280" t="s">
-        <v>1094</v>
+        <v>1089</v>
       </c>
       <c r="K17" s="272" t="s">
-        <v>1136</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="277" t="s">
+        <v>951</v>
+      </c>
+      <c r="B18" s="278" t="s">
+        <v>952</v>
+      </c>
+      <c r="C18" s="278" t="s">
+        <v>953</v>
+      </c>
+      <c r="D18" s="278" t="s">
+        <v>954</v>
+      </c>
+      <c r="E18" s="278" t="s">
+        <v>955</v>
+      </c>
+      <c r="F18" s="278" t="s">
         <v>956</v>
       </c>
-      <c r="B18" s="278" t="s">
+      <c r="H18" s="274" t="s">
         <v>957</v>
       </c>
-      <c r="C18" s="278" t="s">
-        <v>958</v>
-      </c>
-      <c r="D18" s="278" t="s">
-        <v>959</v>
-      </c>
-      <c r="E18" s="278" t="s">
-        <v>960</v>
-      </c>
-      <c r="F18" s="278" t="s">
-        <v>961</v>
-      </c>
-      <c r="H18" s="274" t="s">
-        <v>962</v>
-      </c>
       <c r="J18" s="280" t="s">
-        <v>1095</v>
+        <v>1090</v>
       </c>
       <c r="K18" s="272" t="s">
-        <v>1137</v>
+        <v>1132</v>
       </c>
       <c r="L18" s="272" t="s">
-        <v>1138</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="277" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="B19" s="278" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="C19" s="278" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="D19" s="278" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="E19" s="278" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
       <c r="F19" s="278" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="G19" s="279" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="H19" s="279" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="J19" s="280" t="s">
-        <v>1096</v>
+        <v>1091</v>
       </c>
       <c r="K19" s="272" t="s">
-        <v>1139</v>
+        <v>1134</v>
       </c>
       <c r="L19" s="272" t="s">
-        <v>1140</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="273" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="B20" s="274" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="C20" s="274" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="G20" s="279" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="H20" s="274" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
       <c r="J20" s="280" t="s">
-        <v>1097</v>
+        <v>1092</v>
       </c>
       <c r="K20" s="272" t="s">
-        <v>1141</v>
+        <v>1136</v>
       </c>
       <c r="L20" s="272" t="s">
-        <v>1142</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1">
       <c r="A21" s="277" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="B21" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="C21" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="D21" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="E21" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="G21" s="276" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="H21" s="274" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
       <c r="J21" s="280" t="s">
-        <v>1098</v>
+        <v>1093</v>
       </c>
       <c r="K21" s="272" t="s">
-        <v>1143</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="277" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="B22" s="278" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
       <c r="C22" s="278" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="D22" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="E22" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="F22" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="G22" s="279" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="H22" s="274" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
       <c r="J22" s="280" t="s">
-        <v>1099</v>
+        <v>1094</v>
       </c>
       <c r="K22" s="272" t="s">
-        <v>1144</v>
+        <v>1139</v>
       </c>
       <c r="L22" s="272" t="s">
-        <v>1145</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="277" t="s">
-        <v>983</v>
+        <v>978</v>
       </c>
       <c r="B23" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="C23" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="D23" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="E23" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="F23" s="278" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="G23" s="279" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="H23" s="274" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="J23" s="280" t="s">
-        <v>1100</v>
+        <v>1095</v>
       </c>
       <c r="K23" s="272" t="s">
-        <v>1146</v>
+        <v>1141</v>
       </c>
       <c r="L23" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="277" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="B24" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="C24" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="D24" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E24" s="278" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="H24" s="274" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="J24" s="280" t="s">
-        <v>1101</v>
+        <v>1096</v>
       </c>
       <c r="K24" s="272" t="s">
-        <v>1148</v>
+        <v>1143</v>
       </c>
       <c r="L24" s="272" t="s">
-        <v>1149</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="277" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="B25" s="278">
         <v>0.05</v>
@@ -25355,10 +25333,10 @@
         <v>0.05</v>
       </c>
       <c r="D25" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E25" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G25" s="279">
         <v>0.05</v>
@@ -25367,274 +25345,274 @@
         <v>0.04</v>
       </c>
       <c r="J25" s="280" t="s">
-        <v>1102</v>
+        <v>1097</v>
       </c>
       <c r="K25" s="272" t="s">
-        <v>1150</v>
+        <v>1145</v>
       </c>
       <c r="L25" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="277" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
       <c r="B26" s="278" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="C26" s="278" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
       <c r="D26" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E26" s="278" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
       <c r="G26" s="279" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
       <c r="H26" s="274" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="J26" s="280" t="s">
-        <v>1103</v>
+        <v>1098</v>
       </c>
       <c r="K26" s="272" t="s">
-        <v>1151</v>
+        <v>1146</v>
       </c>
       <c r="L26" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="277" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
       <c r="B27" s="278" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="C27" s="278" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="D27" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E27" s="278" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="H27" s="278" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="J27" s="280" t="s">
-        <v>1104</v>
+        <v>1099</v>
       </c>
       <c r="K27" s="272" t="s">
-        <v>1152</v>
+        <v>1147</v>
       </c>
       <c r="L27" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="277" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="B28" s="278" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="C28" s="278" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="D28" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E28" s="278" t="s">
-        <v>996</v>
+        <v>991</v>
       </c>
       <c r="G28" s="278" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
       <c r="H28" s="274" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="J28" s="280" t="s">
-        <v>1105</v>
+        <v>1100</v>
       </c>
       <c r="K28" s="272" t="s">
-        <v>1153</v>
+        <v>1148</v>
       </c>
       <c r="L28" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="15" customHeight="1">
       <c r="A29" s="277" t="s">
+        <v>993</v>
+      </c>
+      <c r="B29" s="278" t="s">
+        <v>994</v>
+      </c>
+      <c r="C29" s="278" t="s">
+        <v>995</v>
+      </c>
+      <c r="D29" s="278" t="s">
+        <v>996</v>
+      </c>
+      <c r="E29" s="278" t="s">
+        <v>994</v>
+      </c>
+      <c r="G29" s="279" t="s">
+        <v>997</v>
+      </c>
+      <c r="H29" s="274" t="s">
         <v>998</v>
       </c>
-      <c r="B29" s="278" t="s">
-        <v>999</v>
-      </c>
-      <c r="C29" s="278" t="s">
-        <v>1000</v>
-      </c>
-      <c r="D29" s="278" t="s">
-        <v>1001</v>
-      </c>
-      <c r="E29" s="278" t="s">
-        <v>999</v>
-      </c>
-      <c r="G29" s="279" t="s">
-        <v>1002</v>
-      </c>
-      <c r="H29" s="274" t="s">
-        <v>1003</v>
-      </c>
       <c r="J29" s="280" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
       <c r="K29" s="272" t="s">
-        <v>1154</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="277" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="B30" s="278" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="C30" s="278" t="s">
-        <v>1006</v>
+        <v>1001</v>
       </c>
       <c r="D30" s="278" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="E30" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G30" s="279" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="H30" s="274" t="s">
-        <v>1007</v>
+        <v>1002</v>
       </c>
       <c r="J30" s="280" t="s">
-        <v>1107</v>
+        <v>1102</v>
       </c>
       <c r="K30" s="272" t="s">
-        <v>1155</v>
+        <v>1150</v>
       </c>
       <c r="L30" s="272" t="s">
-        <v>1156</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="277" t="s">
-        <v>1008</v>
+        <v>1003</v>
       </c>
       <c r="B31" s="278" t="s">
-        <v>1009</v>
+        <v>1004</v>
       </c>
       <c r="C31" s="278" t="s">
-        <v>1009</v>
+        <v>1004</v>
       </c>
       <c r="D31" s="278" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="E31" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G31" s="279" t="s">
-        <v>1010</v>
+        <v>1005</v>
       </c>
       <c r="H31" s="278" t="s">
-        <v>1009</v>
+        <v>1004</v>
       </c>
       <c r="J31" s="280" t="s">
-        <v>1108</v>
+        <v>1103</v>
       </c>
       <c r="K31" s="272" t="s">
-        <v>1157</v>
+        <v>1152</v>
       </c>
       <c r="L31" s="272" t="s">
-        <v>1158</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="277" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
       <c r="B32" s="278" t="s">
-        <v>1012</v>
+        <v>1007</v>
       </c>
       <c r="C32" s="278" t="s">
-        <v>1012</v>
+        <v>1007</v>
       </c>
       <c r="D32" s="278" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="E32" s="278" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G32" s="279" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
       <c r="H32" s="274" t="s">
-        <v>1014</v>
+        <v>1009</v>
       </c>
       <c r="J32" s="280" t="s">
-        <v>1109</v>
+        <v>1104</v>
       </c>
       <c r="K32" s="272" t="s">
-        <v>1159</v>
+        <v>1154</v>
       </c>
       <c r="L32" s="272" t="s">
-        <v>1160</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="277" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B33" s="278" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C33" s="278" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D33" s="278" t="s">
+        <v>996</v>
+      </c>
+      <c r="E33" s="278" t="s">
+        <v>1013</v>
+      </c>
+      <c r="G33" s="279" t="s">
+        <v>1014</v>
+      </c>
+      <c r="H33" s="274" t="s">
         <v>1015</v>
       </c>
-      <c r="B33" s="278" t="s">
-        <v>1016</v>
-      </c>
-      <c r="C33" s="278" t="s">
-        <v>1017</v>
-      </c>
-      <c r="D33" s="278" t="s">
-        <v>1001</v>
-      </c>
-      <c r="E33" s="278" t="s">
-        <v>1018</v>
-      </c>
-      <c r="G33" s="279" t="s">
-        <v>1019</v>
-      </c>
-      <c r="H33" s="274" t="s">
-        <v>1020</v>
-      </c>
       <c r="J33" s="280" t="s">
-        <v>1110</v>
+        <v>1105</v>
       </c>
       <c r="K33" s="272" t="s">
-        <v>1161</v>
+        <v>1156</v>
       </c>
       <c r="L33" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="277" t="s">
-        <v>1021</v>
+        <v>1016</v>
       </c>
       <c r="B34" s="278" t="s">
-        <v>1022</v>
+        <v>1017</v>
       </c>
       <c r="C34" s="278" t="s">
-        <v>1023</v>
+        <v>1018</v>
       </c>
       <c r="D34" s="278">
         <v>1000</v>
@@ -25652,18 +25630,18 @@
         <v>9800</v>
       </c>
       <c r="J34" s="280" t="s">
-        <v>1111</v>
+        <v>1106</v>
       </c>
       <c r="K34" s="272" t="s">
-        <v>1162</v>
+        <v>1157</v>
       </c>
       <c r="L34" s="272" t="s">
-        <v>1163</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="15" customHeight="1">
       <c r="A35" s="277" t="s">
-        <v>1024</v>
+        <v>1019</v>
       </c>
       <c r="B35" s="278">
         <v>1.75</v>
@@ -25687,158 +25665,158 @@
         <v>1.75</v>
       </c>
       <c r="K35" s="272" t="s">
-        <v>1164</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="36" spans="1:12">
       <c r="K36" s="272" t="s">
-        <v>1165</v>
+        <v>1160</v>
       </c>
       <c r="L36" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="37" spans="1:12">
       <c r="K37" s="272" t="s">
-        <v>1166</v>
+        <v>1161</v>
       </c>
       <c r="L37" s="272" t="s">
-        <v>1167</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="38" spans="1:12">
       <c r="K38" s="272" t="s">
-        <v>1168</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="39" spans="1:12">
       <c r="K39" s="272" t="s">
-        <v>1169</v>
+        <v>1164</v>
       </c>
       <c r="L39" s="272" t="s">
-        <v>1170</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="40" spans="1:12">
       <c r="K40" s="272" t="s">
-        <v>1171</v>
+        <v>1166</v>
       </c>
       <c r="L40" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="41" spans="1:12">
       <c r="K41" s="272" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="L41" s="272" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="42" spans="1:12">
       <c r="K42" s="272" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L42" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="43" spans="1:12">
       <c r="K43" s="272" t="s">
-        <v>1175</v>
+        <v>1170</v>
       </c>
       <c r="L43" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="44" spans="1:12">
       <c r="K44" s="272" t="s">
-        <v>1176</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="45" spans="1:12">
       <c r="K45" s="272" t="s">
-        <v>1177</v>
+        <v>1172</v>
       </c>
       <c r="L45" s="272" t="s">
-        <v>1178</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="46" spans="1:12">
       <c r="K46" s="272" t="s">
-        <v>1179</v>
+        <v>1174</v>
       </c>
       <c r="L46" s="272" t="s">
-        <v>1180</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="47" spans="1:12">
       <c r="K47" s="272" t="s">
-        <v>1181</v>
+        <v>1176</v>
       </c>
       <c r="L47" s="272" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="48" spans="1:12">
       <c r="K48" s="272" t="s">
-        <v>1183</v>
+        <v>1178</v>
       </c>
       <c r="L48" s="272" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="49" spans="11:12">
       <c r="K49" s="272" t="s">
-        <v>1185</v>
+        <v>1180</v>
       </c>
       <c r="L49" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="50" spans="11:12">
       <c r="K50" s="272" t="s">
-        <v>1186</v>
+        <v>1181</v>
       </c>
       <c r="L50" s="272" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="51" spans="11:12">
       <c r="K51" s="272" t="s">
-        <v>1188</v>
+        <v>1183</v>
       </c>
       <c r="L51" s="272" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="52" spans="11:12">
       <c r="K52" s="272" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="53" spans="11:12">
       <c r="K53" s="272" t="s">
-        <v>1190</v>
+        <v>1185</v>
       </c>
       <c r="L53" s="272" t="s">
-        <v>1191</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="54" spans="11:12">
       <c r="K54" s="272" t="s">
-        <v>1192</v>
+        <v>1187</v>
       </c>
       <c r="L54" s="272" t="s">
-        <v>1193</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="55" spans="11:12">
       <c r="K55" s="272" t="s">
-        <v>1194</v>
+        <v>1189</v>
       </c>
       <c r="L55" s="272" t="s">
-        <v>1195</v>
+        <v>1190</v>
       </c>
     </row>
   </sheetData>
@@ -25863,46 +25841,46 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75">
       <c r="A1" s="5" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
       <c r="B1" t="s">
-        <v>1026</v>
+        <v>1021</v>
       </c>
       <c r="C1" t="s">
-        <v>1027</v>
+        <v>1022</v>
       </c>
       <c r="D1" t="s">
-        <v>1028</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>1029</v>
+        <v>1024</v>
       </c>
       <c r="B2" t="s">
-        <v>1030</v>
+        <v>1025</v>
       </c>
       <c r="C2" s="137" t="s">
-        <v>1031</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>1032</v>
+        <v>1027</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1033</v>
+        <v>1028</v>
       </c>
       <c r="C3" s="94" t="s">
-        <v>1031</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>1034</v>
+        <v>1029</v>
       </c>
       <c r="B4" t="s">
-        <v>1035</v>
+        <v>1030</v>
       </c>
       <c r="C4" t="s">
         <v>357</v>
@@ -25910,29 +25888,29 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>1036</v>
+        <v>1031</v>
       </c>
       <c r="B5" t="s">
-        <v>1037</v>
+        <v>1032</v>
       </c>
       <c r="C5" s="149" t="s">
-        <v>1038</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>1039</v>
+        <v>1034</v>
       </c>
       <c r="B6" t="s">
-        <v>1033</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>1040</v>
+        <v>1035</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1041</v>
+        <v>1036</v>
       </c>
     </row>
   </sheetData>
@@ -25957,7 +25935,7 @@
         <v>360</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1042</v>
+        <v>1037</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>361</v>
@@ -25966,12 +25944,12 @@
         <v>7</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>1043</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="139" t="s">
-        <v>1044</v>
+        <v>1039</v>
       </c>
       <c r="B2" s="139"/>
       <c r="C2" s="139"/>
@@ -25980,81 +25958,81 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>1045</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>1046</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>1047</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>1048</v>
+        <v>1043</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>1049</v>
+        <v>1044</v>
       </c>
       <c r="E6" s="99" t="s">
-        <v>1050</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>1051</v>
+        <v>1046</v>
       </c>
       <c r="C7" t="s">
-        <v>1052</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" customHeight="1"/>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>1053</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>1054</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>1055</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>1056</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>1057</v>
+        <v>1052</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>1058</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>1059</v>
+        <v>1054</v>
       </c>
       <c r="C15" t="s">
-        <v>1060</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>1061</v>
+        <v>1056</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -26062,7 +26040,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="4" t="s">
-        <v>1062</v>
+        <v>1057</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -26070,71 +26048,71 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="136" t="s">
-        <v>1063</v>
+        <v>1058</v>
       </c>
       <c r="E19" s="99" t="s">
-        <v>1064</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75">
       <c r="A21" s="140" t="s">
-        <v>1065</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>1066</v>
+        <v>1061</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>1068</v>
+        <v>1063</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="E23" s="99" t="s">
-        <v>1069</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:5" ht="15.75">
       <c r="A29" s="140" t="s">
-        <v>1070</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>1071</v>
+        <v>1066</v>
       </c>
       <c r="B30" t="s">
-        <v>1072</v>
+        <v>1067</v>
       </c>
       <c r="C30" t="s">
-        <v>1073</v>
+        <v>1068</v>
       </c>
       <c r="D30" t="s">
-        <v>1074</v>
+        <v>1069</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>1075</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75">
       <c r="A31" s="138" t="s">
-        <v>1076</v>
+        <v>1071</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="E31" t="s">
-        <v>1077</v>
+        <v>1072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>